<commit_message>
Added some new functionality
</commit_message>
<xml_diff>
--- a/quiz_questions.xlsx
+++ b/quiz_questions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/craigmarkowitz/Documents/Development/Claude Apps/music-iq-claude-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1C6CC196-5BF4-AA4D-AD81-1505165257FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{601DE1F1-69C8-2E46-81E9-1425CBB752C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="35840" windowHeight="19880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="35840" windowHeight="19880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Music Knowledge" sheetId="1" r:id="rId1"/>
@@ -2707,6 +2707,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">

</xml_diff>